<commit_message>
Add Textainer tracking, PIL parser, and fix Maersk tracking number validation
</commit_message>
<xml_diff>
--- a/Major_Shipping_Line_Tracking_URLsMyChanges.xlsx
+++ b/Major_Shipping_Line_Tracking_URLsMyChanges.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BrijeshVerma\Desktop\XPortPlusWebsite\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1DD7211-0F51-4A21-ADEA-121134C13886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{370D399A-C9AA-4262-B429-605D31E7EB92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -403,7 +403,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -503,8 +503,16 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -537,18 +545,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF7030A0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="3" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -556,12 +552,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -607,34 +597,24 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -645,10 +625,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -669,7 +649,10 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -994,27 +977,27 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="2" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="24" t="s">
         <v>39</v>
       </c>
       <c r="F2" t="s">
@@ -1022,19 +1005,19 @@
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="E3" s="8" t="s">
+      <c r="D3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>38</v>
       </c>
       <c r="F3" t="s">
@@ -1042,53 +1025,53 @@
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="41" t="s">
+      <c r="D4" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="41" t="s">
+      <c r="E4" s="6" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="34" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E6" s="7" t="s">
+      <c r="D6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>48</v>
       </c>
       <c r="F6" t="s">
@@ -1096,56 +1079,56 @@
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" s="7" t="s">
+      <c r="D7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="26" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="E8" s="16" t="s">
+      <c r="D8" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="30" t="s">
+      <c r="B9" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E9" s="32" t="s">
+      <c r="D9" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" s="24" t="s">
         <v>97</v>
       </c>
       <c r="F9" t="s">
@@ -1153,36 +1136,36 @@
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E10" s="9" t="s">
+      <c r="D10" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="20" t="s">
+      <c r="B11" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="D11" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E11" s="7" t="s">
+      <c r="D11" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>43</v>
       </c>
       <c r="F11" t="s">
@@ -1190,19 +1173,19 @@
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="20" t="s">
+      <c r="B12" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="D12" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" s="7" t="s">
+      <c r="D12" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>38</v>
       </c>
       <c r="F12" t="s">
@@ -1210,289 +1193,289 @@
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="29" t="s">
+      <c r="A13" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="30" t="s">
+      <c r="B13" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="C13" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="D13" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E13" s="7" t="s">
+      <c r="D13" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="D14" s="16" t="s">
+      <c r="D14" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="E14" s="16" t="s">
+      <c r="E14" s="5" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="29" t="s">
+      <c r="A15" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="30" t="s">
+      <c r="B15" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="29" t="s">
+      <c r="C15" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="D15" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E15" s="7" t="s">
+      <c r="D15" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="27" t="s">
+      <c r="A16" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="28" t="s">
+      <c r="B16" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="C16" s="27" t="s">
+      <c r="C16" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="D16" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E16" s="7" t="s">
+      <c r="D16" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="24" t="s">
+      <c r="A17" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="B17" s="31" t="s">
+      <c r="B17" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="C17" s="24" t="s">
+      <c r="C17" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="D17" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="E17" s="14" t="s">
+      <c r="D17" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E17" s="33" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="21" t="s">
+      <c r="B18" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D18" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="E18" s="11" t="s">
+      <c r="D18" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E18" s="7" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="21" t="s">
+      <c r="A19" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="B19" s="21" t="s">
+      <c r="B19" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="C19" s="21" t="s">
+      <c r="C19" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D19" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="E19" s="11" t="s">
+      <c r="D19" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E19" s="7" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="D20" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="E20" s="15" t="s">
+      <c r="D20" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E20" s="8" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="B21" s="21" t="s">
+      <c r="B21" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="C21" s="21" t="s">
+      <c r="C21" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D21" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="E21" s="11" t="s">
+      <c r="D21" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E21" s="7" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="29">
-      <c r="A22" s="24" t="s">
+      <c r="A22" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="B22" s="24" t="s">
+      <c r="B22" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="C22" s="24" t="s">
+      <c r="C22" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="D22" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="E22" s="14" t="s">
+      <c r="D22" s="33" t="s">
+        <v>36</v>
+      </c>
+      <c r="E22" s="33" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="24" t="s">
+      <c r="A23" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="B23" s="24" t="s">
+      <c r="B23" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="C23" s="24" t="s">
+      <c r="C23" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="D23" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="E23" s="12" t="s">
+      <c r="D23" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E23" s="8" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="23" t="s">
+      <c r="A24" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="B24" s="23" t="s">
+      <c r="B24" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="C24" s="23" t="s">
+      <c r="C24" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="D24" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="E24" s="17" t="s">
+      <c r="D24" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E24" s="9" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="29">
-      <c r="A25" s="23" t="s">
+      <c r="A25" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="B25" s="23" t="s">
+      <c r="B25" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="C25" s="23" t="s">
+      <c r="C25" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="D25" s="18"/>
-      <c r="E25" s="17" t="s">
+      <c r="D25" s="10"/>
+      <c r="E25" s="9" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="29">
-      <c r="A26" s="21" t="s">
+      <c r="A26" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="B26" s="21" t="s">
+      <c r="B26" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="C26" s="21" t="s">
+      <c r="C26" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D26" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="E26" s="11" t="s">
+      <c r="D26" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E26" s="7" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="29">
-      <c r="A27" s="21" t="s">
+      <c r="A27" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="B27" s="21" t="s">
+      <c r="B27" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="C27" s="21" t="s">
+      <c r="C27" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D27" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="E27" s="11" t="s">
+      <c r="D27" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E27" s="7" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="23" t="s">
+      <c r="A28" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="B28" s="23" t="s">
+      <c r="B28" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="C28" s="23" t="s">
+      <c r="C28" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="D28" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="E28" s="18" t="s">
+      <c r="D28" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="E28" s="10" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="29">
-      <c r="A29" s="21" t="s">
+      <c r="A29" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="B29" s="21" t="s">
+      <c r="B29" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="C29" s="21" t="s">
+      <c r="C29" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D29" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="E29" s="8" t="s">
+      <c r="D29" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E29" s="4" t="s">
         <v>84</v>
       </c>
       <c r="F29" t="s">
@@ -1500,90 +1483,90 @@
       </c>
     </row>
     <row r="30" spans="1:6">
-      <c r="A30" s="22" t="s">
+      <c r="A30" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="B30" s="21" t="s">
+      <c r="B30" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="C30" s="21" t="s">
+      <c r="C30" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D30" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="E30" s="8" t="s">
+      <c r="D30" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E30" s="4" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="29">
-      <c r="A31" s="22" t="s">
+      <c r="A31" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="B31" s="21" t="s">
+      <c r="B31" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="C31" s="21" t="s">
+      <c r="C31" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D31" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="E31" s="8" t="s">
+      <c r="D31" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E31" s="4" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="29">
-      <c r="A32" s="22" t="s">
+      <c r="A32" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="B32" s="21" t="s">
+      <c r="B32" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="C32" s="21" t="s">
+      <c r="C32" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D32" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="E32" s="8" t="s">
+      <c r="D32" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E32" s="4" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="18.5">
-      <c r="A36" s="33" t="s">
+      <c r="A36" s="25" t="s">
         <v>98</v>
       </c>
-      <c r="B36" s="34" t="s">
+      <c r="B36" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="C36" s="35" t="s">
+      <c r="C36" s="27" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="41">
-      <c r="A39" s="36" t="s">
+      <c r="A39" s="28" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="40" spans="1:3">
-      <c r="A40" s="37"/>
+      <c r="A40" s="29"/>
     </row>
     <row r="41" spans="1:3">
-      <c r="A41" s="38" t="s">
+      <c r="A41" s="30" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="42" spans="1:3">
-      <c r="A42" s="39"/>
+      <c r="A42" s="31"/>
     </row>
     <row r="43" spans="1:3" ht="52.5">
-      <c r="A43" s="40" t="s">
+      <c r="A43" s="32" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="31.5">
-      <c r="A44" s="40" t="s">
+      <c r="A44" s="32" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1622,5 +1605,6 @@
     <hyperlink ref="B32" r:id="rId31" tooltip="https://www.cnc-line.com/ebusiness/tracking" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId32"/>
 </worksheet>
 </file>
</xml_diff>